<commit_message>
Add Chinese-first auto translation flow
</commit_message>
<xml_diff>
--- a/data/cases.xlsx
+++ b/data/cases.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cases" sheetId="1" r:id="Rddbe81fe268f4516"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="2" r:id="R9e0b3abacc3e4664"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cases" sheetId="1" r:id="Ree227d5da2164b74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="2" r:id="Rc98b8d70d4c6496f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -497,13 +497,13 @@
         <x:v>luma-moonbun</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>Luma</x:v>
+        <x:v>露玛</x:v>
       </x:c>
       <x:c r="C2" s="7" t="str">
-        <x:v>Moonbun</x:v>
+        <x:v>月兔团</x:v>
       </x:c>
       <x:c r="D2" s="7" t="str">
-        <x:v>soft ache</x:v>
+        <x:v>柔软的难过</x:v>
       </x:c>
       <x:c r="E2" s="7" t="str">
         <x:v>#f3bc88</x:v>
@@ -515,22 +515,22 @@
         <x:v>listen</x:v>
       </x:c>
       <x:c r="H2" s="7" t="str">
-        <x:v>Luma keeps dreaming of a ladder made of moonlight. Every step breaks before the top.</x:v>
+        <x:v>露玛总是梦见一架月光做成的梯子。每爬到快要够着月亮时，下一阶就碎掉了。</x:v>
       </x:c>
       <x:c r="I2" s="7" t="str">
-        <x:v>The nightmare smells like warm milk and old paper.</x:v>
+        <x:v>噩梦闻起来像温热的牛奶和旧信纸。</x:v>
       </x:c>
       <x:c r="J2" s="7" t="str">
-        <x:v>Luma says the moon never answers letters.</x:v>
+        <x:v>露玛说月亮从来不回信。</x:v>
       </x:c>
       <x:c r="K2" s="7" t="str">
-        <x:v>A tiny envelope is tucked under one paw.</x:v>
+        <x:v>一只小信封压在她的爪子下面。</x:v>
       </x:c>
       <x:c r="L2" s="7" t="str">
-        <x:v>A moonlit mailbox that rings once, even when the answer is still far away.</x:v>
+        <x:v>诊所送给她一只月光邮箱，就算答案还很远，也会轻轻响一声。</x:v>
       </x:c>
       <x:c r="M2" s="7" t="str">
-        <x:v>Tomorrow, Luma will write the first real letter instead of waiting for the perfect one.</x:v>
+        <x:v>明天，露玛会先写出第一封真正的信，而不是继续等一封完美的信。</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="64" customHeight="1">
@@ -538,13 +538,13 @@
         <x:v>mori-mossfox</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
-        <x:v>Mori</x:v>
+        <x:v>森森</x:v>
       </x:c>
       <x:c r="C3" s="7" t="str">
-        <x:v>Moss Fox</x:v>
+        <x:v>苔狐</x:v>
       </x:c>
       <x:c r="D3" s="7" t="str">
-        <x:v>quiet regret</x:v>
+        <x:v>安静的遗憾</x:v>
       </x:c>
       <x:c r="E3" s="7" t="str">
         <x:v>#91d79b</x:v>
@@ -556,22 +556,22 @@
         <x:v>soothe</x:v>
       </x:c>
       <x:c r="H3" s="7" t="str">
-        <x:v>Mori's dream forest loops forever. A friend keeps waving from the path he did not take.</x:v>
+        <x:v>森森的梦里有一片走不出去的森林。没来得及告别的朋友，总在另一条小路尽头朝他挥手。</x:v>
       </x:c>
       <x:c r="I3" s="7" t="str">
-        <x:v>The same leaf falls every twelve seconds.</x:v>
+        <x:v>同一片叶子每十二秒落下一次。</x:v>
       </x:c>
       <x:c r="J3" s="7" t="str">
-        <x:v>Mori apologizes before anyone speaks.</x:v>
+        <x:v>森森总是在别人开口前先道歉。</x:v>
       </x:c>
       <x:c r="K3" s="7" t="str">
-        <x:v>A seed glows whenever the dream turns backward.</x:v>
+        <x:v>有一粒种子会在梦倒退时发光。</x:v>
       </x:c>
       <x:c r="L3" s="7" t="str">
-        <x:v>A clearing where the missed goodbye can be spoken without the forest ending.</x:v>
+        <x:v>诊所为他开出一片空地，让那句迟到的告别终于可以被说完。</x:v>
       </x:c>
       <x:c r="M3" s="7" t="str">
-        <x:v>Mori wakes with one seed to plant beside the old road.</x:v>
+        <x:v>醒来后，森森会把那粒种子种在旧路旁边。</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="64" customHeight="1">
@@ -579,13 +579,13 @@
         <x:v>nini-glass-hamster</x:v>
       </x:c>
       <x:c r="B4" s="7" t="str">
-        <x:v>Nini</x:v>
+        <x:v>妮妮</x:v>
       </x:c>
       <x:c r="C4" s="7" t="str">
-        <x:v>Glass Hamster</x:v>
+        <x:v>玻璃仓鼠</x:v>
       </x:c>
       <x:c r="D4" s="7" t="str">
-        <x:v>sharp dream</x:v>
+        <x:v>刺人的梦</x:v>
       </x:c>
       <x:c r="E4" s="7" t="str">
         <x:v>#9fd8ff</x:v>
@@ -597,22 +597,22 @@
         <x:v>bottle</x:v>
       </x:c>
       <x:c r="H4" s="7" t="str">
-        <x:v>Nini is transparent tonight. A dark little storm keeps tapping from inside her chest.</x:v>
+        <x:v>妮妮今晚几乎是透明的。胸口里有一小团黑雨，一直敲着玻璃。</x:v>
       </x:c>
       <x:c r="I4" s="7" t="str">
-        <x:v>The storm grows louder when the room is silent.</x:v>
+        <x:v>房间越安静，雨声越大。</x:v>
       </x:c>
       <x:c r="J4" s="7" t="str">
-        <x:v>Nini laughs whenever she is about to cry.</x:v>
+        <x:v>妮妮快哭的时候，总会先笑出来。</x:v>
       </x:c>
       <x:c r="K4" s="7" t="str">
-        <x:v>Her shadow is trying to hide under the clipboard.</x:v>
+        <x:v>她的影子躲在病历夹下面。</x:v>
       </x:c>
       <x:c r="L4" s="7" t="str">
-        <x:v>A corked rain bottle, small enough to hold and safe enough to open later.</x:v>
+        <x:v>诊所把黑雨收进一只带软木塞的小瓶，等她准备好时再慢慢打开。</x:v>
       </x:c>
       <x:c r="M4" s="7" t="str">
-        <x:v>Nini learns she can name a feeling before it fills the whole room.</x:v>
+        <x:v>明天，妮妮会先说出一个感受的名字，不让它填满整个房间。</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="64" customHeight="1">
@@ -620,13 +620,13 @@
         <x:v>puff-cloudcat</x:v>
       </x:c>
       <x:c r="B5" s="7" t="str">
-        <x:v>Puff</x:v>
+        <x:v>噗芙</x:v>
       </x:c>
       <x:c r="C5" s="7" t="str">
-        <x:v>Cloud Cat</x:v>
+        <x:v>云猫</x:v>
       </x:c>
       <x:c r="D5" s="7" t="str">
-        <x:v>sky wish</x:v>
+        <x:v>天空愿望</x:v>
       </x:c>
       <x:c r="E5" s="7" t="str">
         <x:v>#f4f1ff</x:v>
@@ -638,22 +638,22 @@
         <x:v>listen</x:v>
       </x:c>
       <x:c r="H5" s="7" t="str">
-        <x:v>Puff wants wings, but every dream flight ends with the city lights drifting away.</x:v>
+        <x:v>噗芙想要一对翅膀，可每次飞起来，城市的灯都会离她越来越远。</x:v>
       </x:c>
       <x:c r="I5" s="7" t="str">
-        <x:v>The wind chime only rings when Puff looks down.</x:v>
+        <x:v>风铃只在她低头时响。</x:v>
       </x:c>
       <x:c r="J5" s="7" t="str">
-        <x:v>Pawprints appear on the ceiling.</x:v>
+        <x:v>天花板上出现了一串爪印。</x:v>
       </x:c>
       <x:c r="K5" s="7" t="str">
-        <x:v>Puff whispers that roofs are almost skies.</x:v>
+        <x:v>噗芙小声说，屋顶几乎就是天空。</x:v>
       </x:c>
       <x:c r="L5" s="7" t="str">
-        <x:v>One safe flight over the rooftops, with every window glowing hello.</x:v>
+        <x:v>诊所送她一场安全的屋顶飞行，每扇窗都亮着欢迎她回来。</x:v>
       </x:c>
       <x:c r="M5" s="7" t="str">
-        <x:v>Puff decides to climb to the roof tomorrow and watch the sunrise from there.</x:v>
+        <x:v>明天，噗芙会爬上屋顶，看一次真正的日出。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="64" customHeight="1">
@@ -661,13 +661,13 @@
         <x:v>fenn-lanterndeer</x:v>
       </x:c>
       <x:c r="B6" s="7" t="str">
-        <x:v>Fenn</x:v>
+        <x:v>芬恩</x:v>
       </x:c>
       <x:c r="C6" s="7" t="str">
-        <x:v>Lantern Deer</x:v>
+        <x:v>灯鹿</x:v>
       </x:c>
       <x:c r="D6" s="7" t="str">
-        <x:v>dim courage</x:v>
+        <x:v>微弱的勇气</x:v>
       </x:c>
       <x:c r="E6" s="7" t="str">
         <x:v>#ffd26f</x:v>
@@ -679,22 +679,22 @@
         <x:v>soothe</x:v>
       </x:c>
       <x:c r="H6" s="7" t="str">
-        <x:v>Fenn's lantern goes out whenever the dream asks him to step onto a stage.</x:v>
+        <x:v>梦一要求芬恩走上舞台，他角上的小灯就会灭掉。</x:v>
       </x:c>
       <x:c r="I6" s="7" t="str">
-        <x:v>Tiny applause hides inside the lantern glass.</x:v>
+        <x:v>灯罩里藏着很小很小的掌声。</x:v>
       </x:c>
       <x:c r="J6" s="7" t="str">
-        <x:v>Fenn knows the song but not the first note.</x:v>
+        <x:v>芬恩记得整首歌，却找不到第一个音。</x:v>
       </x:c>
       <x:c r="K6" s="7" t="str">
-        <x:v>The nightmare is brightest just before he begins.</x:v>
+        <x:v>噩梦总在他准备开始前变得最亮。</x:v>
       </x:c>
       <x:c r="L6" s="7" t="str">
-        <x:v>A stage where the first note can tremble and still count.</x:v>
+        <x:v>诊所为他点亮一座允许颤抖的舞台，第一声跑调也算数。</x:v>
       </x:c>
       <x:c r="M6" s="7" t="str">
-        <x:v>Fenn wakes ready to sing badly once, which is how songs begin.</x:v>
+        <x:v>明天，芬恩会先唱坏一次，因为歌就是这样开始的。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="64" customHeight="1">
@@ -702,13 +702,13 @@
         <x:v>no7-unknown-kit</x:v>
       </x:c>
       <x:c r="B7" s="8" t="str">
-        <x:v>No. 7</x:v>
+        <x:v>七号</x:v>
       </x:c>
       <x:c r="C7" s="8" t="str">
-        <x:v>Unknown Kit</x:v>
+        <x:v>未知幼兽</x:v>
       </x:c>
       <x:c r="D7" s="8" t="str">
-        <x:v>sealed fear</x:v>
+        <x:v>封住的害怕</x:v>
       </x:c>
       <x:c r="E7" s="8" t="str">
         <x:v>#ff9aa2</x:v>
@@ -720,22 +720,22 @@
         <x:v>bottle</x:v>
       </x:c>
       <x:c r="H7" s="8" t="str">
-        <x:v>No. 7 arrives with no name tag. The dream door behind them locks itself twice.</x:v>
+        <x:v>七号没有名字牌。她身后的梦门自己上了两道锁。</x:v>
       </x:c>
       <x:c r="I7" s="8" t="str">
-        <x:v>The nightmare repeats your last sentence in a smaller voice.</x:v>
+        <x:v>噩梦会用更小的声音重复你上一句话。</x:v>
       </x:c>
       <x:c r="J7" s="8" t="str">
-        <x:v>No. 7 flinches when called monster.</x:v>
+        <x:v>有人叫她怪物时，七号会立刻缩起来。</x:v>
       </x:c>
       <x:c r="K7" s="8" t="str">
-        <x:v>A blank collar waits beside the dream door.</x:v>
+        <x:v>一枚空白项圈放在梦门旁边。</x:v>
       </x:c>
       <x:c r="L7" s="8" t="str">
-        <x:v>A quiet room where the word monster turns back into the word scared.</x:v>
+        <x:v>诊所给她一间安静房间，让怪物这个词慢慢变回害怕。</x:v>
       </x:c>
       <x:c r="M7" s="8" t="str">
-        <x:v>No. 7 leaves with a blank tag and permission to choose a name later.</x:v>
+        <x:v>七号带着空白名字牌离开，她可以晚一点再决定自己叫什么。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="64" customHeight="1"/>

</xml_diff>